<commit_message>
Update Contracts test cases - 23130094
</commit_message>
<xml_diff>
--- a/Group03_23130094_BuiAnhHau.xlsx
+++ b/Group03_23130094_BuiAnhHau.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="274">
   <si>
     <t xml:space="preserve">TEST CASE</t>
   </si>
@@ -589,9 +589,6 @@
   </si>
   <si>
     <t xml:space="preserve">1. New contract screen is displayed (page title = "New contract")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026</t>
   </si>
   <si>
     <t xml:space="preserve">PRE: Signed in the Dolibarr demo with the Contracts module enabled; at least 1 Third party exists.
@@ -608,9 +605,6 @@
     - Buttons [CREATE DRAFT] and [CANCEL]</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026. Demo còn có trường "aaa" (Automatically calculated) - trường tùy chỉnh, không kiểm tra</t>
-  </si>
-  <si>
     <t xml:space="preserve">Check creating a draft contract with only the required field (Third party)</t>
   </si>
   <si>
@@ -624,9 +618,6 @@
     - Status = Draft
     - Ref is a provisional ref (e.g. "(PROV...)")
     - Third party = Testldr1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026: tạo được hợp đồng (PROV24), Status Draft, Third party Testldr1</t>
   </si>
   <si>
     <t xml:space="preserve">Check creating a contract with Note (internal) filled</t>
@@ -643,9 +634,6 @@
 4. Tab [Notes] shows the internal note = "Internal note 01"</t>
   </si>
   <si>
-    <t xml:space="preserve">Ô Note (public) là trình soạn thảo rich text, khó record nên chỉ nhập Note (internal)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Check required field - Third party</t>
   </si>
   <si>
@@ -657,9 +645,6 @@
     <t xml:space="preserve">2. New contract screen is still displayed
     - Error message "Field 'Third party' is required" is displayed
     - No contract is created</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026: thông báo lỗi đỏ hiện ở góc trên bên phải</t>
   </si>
   <si>
     <t xml:space="preserve">PRE: Signed in the Dolibarr demo with the Contracts module enabled; at least 1 Third party exists. Third party = Testldr1.
@@ -718,9 +703,6 @@
     - Contract date = 01/01/2026 is displayed on Contract detail screen</t>
   </si>
   <si>
-    <t xml:space="preserve">Ngày hiển thị theo định dạng MM/DD/YYYY của bản demo</t>
-  </si>
-  <si>
     <t xml:space="preserve">ADD_CONTRACT-10</t>
   </si>
   <si>
@@ -748,9 +730,6 @@
     - Contract is created and Contract detail screen is displayed</t>
   </si>
   <si>
-    <t xml:space="preserve">Kiểm tra khả năng chịu dữ liệu dài; ghi lại hành vi thực tế (có cắt ký tự hay không)</t>
-  </si>
-  <si>
     <t xml:space="preserve">LIST_CONTRACT</t>
   </si>
   <si>
@@ -768,9 +747,6 @@
     - Table of contracts is displayed</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026: Passed</t>
-  </si>
-  <si>
     <t xml:space="preserve">PRE: Signed in the Dolibarr demo with the Contracts module enabled; at least 1 Third party exists.
 1. Open Contracts list screen (LIST_CONTRACT-01)
 2. Check the columns, the filter row and the icons</t>
@@ -782,9 +758,6 @@
     - Rows of contracts below</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026. Demo có thêm cột "aaa" (trường tùy chỉnh của bản demo, hiển thị lỗi) - không đưa vào Expected</t>
-  </si>
-  <si>
     <t xml:space="preserve">Check searching contracts by an existing Ref</t>
   </si>
   <si>
@@ -833,9 +806,6 @@
     <t xml:space="preserve">3. All displayed contracts have Status = Draft</t>
   </si>
   <si>
-    <t xml:space="preserve">Ô Status nằm bên phải bảng; nếu khó thao tác/record thì đánh dấu Skipped</t>
-  </si>
-  <si>
     <t xml:space="preserve">Check clearing the filter</t>
   </si>
   <si>
@@ -883,9 +853,6 @@
     - Third party is the same as in the list</t>
   </si>
   <si>
-    <t xml:space="preserve">Demo dùng chung có thể reset; nếu không còn CT2610-0007 thì chọn contract đầu tiên trong danh sách</t>
-  </si>
-  <si>
     <t xml:space="preserve">Check going back to the list from Contract detail screen</t>
   </si>
   <si>
@@ -894,9 +861,6 @@
   </si>
   <si>
     <t xml:space="preserve">1. Contracts list screen is displayed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026: link Back to list ở góc trên bên phải trang chi tiết</t>
   </si>
   <si>
     <t xml:space="preserve">EDIT_CONTRACT</t>
@@ -916,9 +880,6 @@
 4. Ref. customer = RC_EDIT_01 is displayed on Contract detail screen</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026: sửa Ref. customer thành RC_EDIT_01 bằng biểu tượng bút chì</t>
-  </si>
-  <si>
     <t xml:space="preserve">Check cancelling modify Ref. customer</t>
   </si>
   <si>
@@ -949,9 +910,6 @@
     <t xml:space="preserve">2. A confirmation message is displayed
 3. Back to Contracts list screen
 4. The deleted contract is not displayed in the list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã chạy thực tế ngày 20-Oct-2026. Chỉ xóa hợp đồng nháp do mình tạo (demo dùng chung)</t>
   </si>
   <si>
     <t xml:space="preserve">Check cancelling delete contract</t>
@@ -2707,7 +2665,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Passed")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Failed")</f>
@@ -2715,7 +2673,7 @@
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">F6-E6-D6-B6-A6</f>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Blocked")</f>
@@ -2775,15 +2733,9 @@
       <c r="E9" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G9" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>187</v>
-      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
@@ -2793,97 +2745,77 @@
         <v>57</v>
       </c>
       <c r="C10" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>188</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>189</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G10" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>190</v>
-      </c>
+      <c r="F10" s="8"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>62</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>191</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>193</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G11" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>194</v>
-      </c>
+      <c r="F11" s="8"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="121.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
         <v>65</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>55</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="23"/>
-      <c r="H12" s="9" t="s">
-        <v>198</v>
-      </c>
+      <c r="H12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
         <v>68</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G13" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>202</v>
-      </c>
+      <c r="F13" s="8"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
@@ -2893,10 +2825,10 @@
         <v>70</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>62</v>
@@ -2910,13 +2842,13 @@
         <v>74</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>89</v>
@@ -2930,13 +2862,13 @@
         <v>77</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>62</v>
@@ -2947,38 +2879,36 @@
     </row>
     <row r="17" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>55</v>
       </c>
       <c r="F17" s="8"/>
       <c r="G17" s="23"/>
-      <c r="H17" s="9" t="s">
-        <v>215</v>
-      </c>
+      <c r="H17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>82</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>55</v>
@@ -2989,25 +2919,23 @@
     </row>
     <row r="19" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>84</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>55</v>
       </c>
       <c r="F19" s="8"/>
       <c r="G19" s="23"/>
-      <c r="H19" s="9" t="s">
-        <v>222</v>
-      </c>
+      <c r="H19" s="9"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F9:F996">
@@ -3061,7 +2989,7 @@
         <v>167</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="J2" s="21" t="s">
         <v>169</v>
@@ -3115,7 +3043,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Passed")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Failed")</f>
@@ -3123,7 +3051,7 @@
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">F6-E6-D6-B6-A6</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Blocked")</f>
@@ -3172,24 +3100,18 @@
         <v>89</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="E9" s="8"/>
-      <c r="F9" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G9" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>227</v>
-      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
@@ -3199,88 +3121,70 @@
         <v>91</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G10" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>230</v>
-      </c>
+      <c r="F10" s="8"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="81" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>95</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G11" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>187</v>
-      </c>
+      <c r="F11" s="8"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
         <v>98</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G12" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>187</v>
-      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
         <v>101</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>89</v>
@@ -3294,61 +3198,53 @@
         <v>104</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>89</v>
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="23"/>
-      <c r="H14" s="9" t="s">
-        <v>243</v>
-      </c>
+      <c r="H14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
         <v>107</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G15" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H15" s="9" t="s">
-        <v>187</v>
-      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
         <v>110</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>89</v>
@@ -3362,13 +3258,13 @@
         <v>112</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>89</v>
@@ -3382,48 +3278,40 @@
         <v>115</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>89</v>
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="23"/>
-      <c r="H18" s="9" t="s">
-        <v>256</v>
-      </c>
+      <c r="H18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
         <v>118</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="F19" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G19" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>260</v>
-      </c>
+      <c r="F19" s="8"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="9"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F9:F996">
@@ -3477,7 +3365,7 @@
         <v>167</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="J2" s="21" t="s">
         <v>169</v>
@@ -3531,7 +3419,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Passed")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Failed")</f>
@@ -3539,7 +3427,7 @@
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">F6-E6-D6-B6-A6</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Blocked")</f>
@@ -3588,39 +3476,33 @@
         <v>122</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G9" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>265</v>
-      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="121.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
         <v>125</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>62</v>
@@ -3681,7 +3563,7 @@
         <v>167</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>269</v>
+        <v>256</v>
       </c>
       <c r="J2" s="21" t="s">
         <v>169</v>
@@ -3735,7 +3617,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Passed")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Failed")</f>
@@ -3743,7 +3625,7 @@
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">F6-E6-D6-B6-A6</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">COUNTIF(F9:F996,"Blocked")</f>
@@ -3792,39 +3674,33 @@
         <v>129</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>272</v>
+        <v>259</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="G9" s="23" t="n">
-        <v>46315</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>273</v>
-      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
         <v>132</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>62</v>
@@ -3878,7 +3754,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="11" t="s">
-        <v>277</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3913,7 +3789,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>278</v>
+        <v>264</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>9</v>
@@ -3924,7 +3800,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>279</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3932,13 +3808,13 @@
         <v>27</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>280</v>
+        <v>266</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>281</v>
+        <v>267</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>282</v>
+        <v>268</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>174</v>
@@ -3950,7 +3826,7 @@
         <v>175</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>283</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3963,7 +3839,7 @@
       </c>
       <c r="D11" s="8" t="n">
         <f aca="false">'Add Contract'!A6</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E11" s="8" t="n">
         <f aca="false">'Add Contract'!B6</f>
@@ -3971,7 +3847,7 @@
       </c>
       <c r="F11" s="8" t="n">
         <f aca="false">'Add Contract'!C6</f>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G11" s="8" t="n">
         <f aca="false">'Add Contract'!D6</f>
@@ -3996,7 +3872,7 @@
       </c>
       <c r="D12" s="8" t="n">
         <f aca="false">'List Contract'!A6</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E12" s="8" t="n">
         <f aca="false">'List Contract'!B6</f>
@@ -4004,7 +3880,7 @@
       </c>
       <c r="F12" s="8" t="n">
         <f aca="false">'List Contract'!C6</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G12" s="8" t="n">
         <f aca="false">'List Contract'!D6</f>
@@ -4029,7 +3905,7 @@
       </c>
       <c r="D13" s="8" t="n">
         <f aca="false">'Edit Contract'!A6</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="8" t="n">
         <f aca="false">'Edit Contract'!B6</f>
@@ -4037,7 +3913,7 @@
       </c>
       <c r="F13" s="8" t="n">
         <f aca="false">'Edit Contract'!C6</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="8" t="n">
         <f aca="false">'Edit Contract'!D6</f>
@@ -4062,7 +3938,7 @@
       </c>
       <c r="D14" s="8" t="n">
         <f aca="false">'Delete Contract'!A6</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="8" t="n">
         <f aca="false">'Delete Contract'!B6</f>
@@ -4070,7 +3946,7 @@
       </c>
       <c r="F14" s="8" t="n">
         <f aca="false">'Delete Contract'!C6</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="8" t="n">
         <f aca="false">'Delete Contract'!D6</f>
@@ -4087,11 +3963,11 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C15" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D15" s="7" t="n">
         <f aca="false">SUM(D11:D14)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
         <f aca="false">SUM(E11:E14)</f>
@@ -4099,7 +3975,7 @@
       </c>
       <c r="F15" s="7" t="n">
         <f aca="false">SUM(F11:F14)</f>
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G15" s="7" t="n">
         <f aca="false">SUM(G11:G14)</f>
@@ -4116,26 +3992,26 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C17" s="2" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="E17" s="24" t="n">
         <f aca="false">IFERROR((D15+E15)*100/(I15-G15-H15),0)</f>
-        <v>46.1538461538462</v>
+        <v>0</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="2" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="E18" s="24" t="n">
         <f aca="false">IFERROR(D15*100/(D15+E15),0)</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>